<commit_message>
more work on css, implements spreadsheet more
</commit_message>
<xml_diff>
--- a/content/timeline.xlsx
+++ b/content/timeline.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55CEEEC3-E2C3-134B-8E9D-5D50D1D8E4FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{017DE8CE-787D-F941-8F80-52C77A37F755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="timeline" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029" concurrentCalc="0"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
   <si>
     <t>class</t>
   </si>
@@ -56,28 +56,95 @@
     <t>timeline-1</t>
   </si>
   <si>
-    <t>Lorem Ipsum</t>
-  </si>
-  <si>
-    <t>timeline-2</t>
-  </si>
-  <si>
-    <t>Dolor sit</t>
-  </si>
-  <si>
-    <t>Title example lol</t>
+    <t>Before Nosgoth's Recorded History</t>
+  </si>
+  <si>
+    <t>subtitle</t>
+  </si>
+  <si>
+    <t>The Wheel of Fate</t>
+  </si>
+  <si>
+    <t>The Land of Nosgoth – ruled by the two elder races, similar in power, but different in method and intention: the Vampires, and the Hylden.</t>
+  </si>
+  <si>
+    <t>The Vampires start worshipping the &lt;b&gt;Wheel of Fate&lt;/b&gt;; a god that represents the cleansing agony of birth, death, and rebirth, the purifying rhythm of the universe – the cycle which sustains all life, to which all souls are irresistibly drawn, manipulated by the parasitic Elder God.</t>
+  </si>
+  <si>
+    <t>The Vampire-Hylden War</t>
+  </si>
+  <si>
+    <t>The Hylden oppose the Vampires’ tyrannous God, and refuse to submit to the Wheel of Fate. For this, the Vampires oppress their Hylden adversaries.</t>
+  </si>
+  <si>
+    <t>The races battle for dominance of Nosgoth in a great, apocalyptic war, which flames for a thousand years, and will destroy both victor and vanquished alike.</t>
+  </si>
+  <si>
+    <t>The Genesis of the Pillars of Nosgoth</t>
+  </si>
+  <si>
+    <t>In triumph, the Vampires banish the Hylden from the world with powerful magic, sealing them into another plane of existence, and raise the Pillars of Nosgoth as the lock that binds them.</t>
+  </si>
+  <si>
+    <t>The nine Pillars reach high into the skies, and deep into the earth (representing Mind, Dimension, Conflict, Nature, Energy, Time, States, Death, and – at the center of all of them binding them together – Balance), intrinsically and supernaturally tied to the spiritual and physical 'health' of the Land.</t>
+  </si>
+  <si>
+    <t>The Summoning of the Guardians</t>
+  </si>
+  <si>
+    <t>With the appointment of the original Vampire Guardians, the Circle of Nine – a body of sorcerers entrusted with the safekeeping of the Pillars – is formed. When a member dies, the supernatural force behind the Pillars culls a worthy successor, who is destined from birth to fulfill that role. &lt;br&gt;&lt;br&gt; Each Guardian is aligned to the principle of the Pillar he serves, and the Balance Guardian is the axis of them all.</t>
+  </si>
+  <si>
+    <t>The Blood Curse</t>
+  </si>
+  <si>
+    <t>In their defeat, the Hylden retaliate as they fall – afflicting the Vampires not only with a predatory blood-thirst, but with sterility as well</t>
+  </si>
+  <si>
+    <t>With the Vampires’ transformation comes their enemies’ true revenge: immortality. Expelled from the cycle of death and rebirth, the apostates are cast from the Wheel of Fate.</t>
+  </si>
+  <si>
+    <t>Plunged into despair, and unable to bear the separation from their God, many Vampires are driven to madness and self-annihilation.</t>
+  </si>
+  <si>
+    <t>The Forging of the Reaver</t>
+  </si>
+  <si>
+    <t>The human Vorador is born</t>
+  </si>
+  <si>
+    <t>The mystical sword known as the Blood Reaver is forged. Imbued with it's maker's lust for blood.</t>
+  </si>
+  <si>
+    <t>The Dark Gift is Passed</t>
+  </si>
+  <si>
+    <t>Vorador is turned; he becomes a vampire</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -101,8 +168,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,13 +506,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="138.6640625" customWidth="1"/>
+    <col min="6" max="6" width="138.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -451,64 +520,208 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="b">
         <v>1</v>
       </c>
-      <c r="C2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="b">
-        <v>0</v>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="F10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="F13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
further additions to code
</commit_message>
<xml_diff>
--- a/content/timeline.xlsx
+++ b/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{017DE8CE-787D-F941-8F80-52C77A37F755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{025D4AD4-E404-384C-84B7-23DCA8C47AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
   <si>
     <t>class</t>
   </si>
@@ -80,9 +80,6 @@
     <t>The races battle for dominance of Nosgoth in a great, apocalyptic war, which flames for a thousand years, and will destroy both victor and vanquished alike.</t>
   </si>
   <si>
-    <t>The Genesis of the Pillars of Nosgoth</t>
-  </si>
-  <si>
     <t>In triumph, the Vampires banish the Hylden from the world with powerful magic, sealing them into another plane of existence, and raise the Pillars of Nosgoth as the lock that binds them.</t>
   </si>
   <si>
@@ -120,6 +117,30 @@
   </si>
   <si>
     <t>Vorador is turned; he becomes a vampire</t>
+  </si>
+  <si>
+    <t>image</t>
+  </si>
+  <si>
+    <t>timeline-1 detail</t>
+  </si>
+  <si>
+    <t>Millennia pass – at least 2,000 years</t>
+  </si>
+  <si>
+    <t>Nosgoth's vampire population increases</t>
+  </si>
+  <si>
+    <t>Nosgoth's early history</t>
+  </si>
+  <si>
+    <t>Over 500 years before Blood Omen: Legacy of Kain</t>
+  </si>
+  <si>
+    <t>Genesis of the Pillars of Nosgoth</t>
+  </si>
+  <si>
+    <t>The formation of the Sarafan (a monastic order of warrior-priests, charged with the eradication of the vampires) by the Circle and the crusade to counter the "vampire menace". Malek commands the armies.</t>
   </si>
 </sst>
 </file>
@@ -506,13 +527,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="138.6640625" customWidth="1"/>
+    <col min="7" max="7" width="138.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -529,199 +550,245 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="F10" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>5</v>
-      </c>
-      <c r="F11" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" s="1" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
-      <c r="F13" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" s="1" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>5</v>
-      </c>
-      <c r="F15" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="F16" s="2" t="s">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>5</v>
-      </c>
-      <c r="F17" s="2" t="s">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="b">
+        <v>1</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" s="1" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>5</v>
-      </c>
-      <c r="F19" s="2" t="s">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="F20" s="2" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" t="b">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" s="1" t="s">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>27</v>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>28</v>
+      </c>
+      <c r="G25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G26" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+      <c r="G27" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
further updates to code - adds data entry to rows to better distinguish what game the event takes place in
</commit_message>
<xml_diff>
--- a/content/timeline.xlsx
+++ b/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C395A97D-850E-C440-9867-85B55E801952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{CD360685-54F8-B545-8DB8-BE15B30DE299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="60">
   <si>
     <t>class</t>
   </si>
@@ -149,9 +149,6 @@
     <t>The Slaughter of the Circle</t>
   </si>
   <si>
-    <t>Janos Audron is excecuted and his heart ripped from his body</t>
-  </si>
-  <si>
     <t>Raziel is born, and becomes a Sarafan warrior-priest</t>
   </si>
   <si>
@@ -191,7 +188,34 @@
     <t>timeline-1 time-travel tt1</t>
   </si>
   <si>
-    <t>#BO-paradox-1</t>
+    <t xml:space="preserve">timeline-1 time-travel </t>
+  </si>
+  <si>
+    <t>#paradox-1</t>
+  </si>
+  <si>
+    <t>Kain discovers another Time Streaming Device and returns to Nosgoth's present</t>
+  </si>
+  <si>
+    <t>#travel-2</t>
+  </si>
+  <si>
+    <t>timeline-2a time-travel tt3</t>
+  </si>
+  <si>
+    <t>Raziel arrives to Nosgoth's past and meets Moebius at the Sarafan fortress, now occupied by the Iron Guard, an army that seeks to avenge the Death of William the Just</t>
+  </si>
+  <si>
+    <t>entry</t>
+  </si>
+  <si>
+    <t>BO</t>
+  </si>
+  <si>
+    <t>SR2</t>
+  </si>
+  <si>
+    <t>Janos Audron is executed and his heart ripped from his body</t>
   </si>
 </sst>
 </file>
@@ -578,385 +602,419 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" customWidth="1"/>
-    <col min="8" max="8" width="138.6640625" customWidth="1"/>
+    <col min="1" max="2" width="23.33203125" customWidth="1"/>
+    <col min="9" max="9" width="138.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="b">
+      <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" t="b">
+      <c r="E3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="b">
+      <c r="E6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="D9" t="b">
+      <c r="E9" t="b">
         <v>1</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>5</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>5</v>
       </c>
-      <c r="D12" t="b">
+      <c r="E12" t="b">
         <v>1</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>5</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>5</v>
       </c>
-      <c r="D14" t="b">
+      <c r="E14" t="b">
         <v>1</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>5</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>5</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="I16" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="I17" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>5</v>
       </c>
-      <c r="D18" t="b">
+      <c r="E18" t="b">
         <v>1</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>5</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>5</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="I20" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>5</v>
       </c>
-      <c r="D21" t="b">
+      <c r="E21" t="b">
         <v>1</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>5</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="I22" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>28</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="I23" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>5</v>
       </c>
-      <c r="C24" t="b">
+      <c r="D24" t="b">
         <v>1</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="I24" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>28</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>5</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>5</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>5</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>5</v>
+      </c>
+      <c r="I29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>5</v>
+      </c>
+      <c r="I31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>5</v>
+      </c>
+      <c r="I32" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>5</v>
-      </c>
-      <c r="H29" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" t="b">
-        <v>1</v>
-      </c>
-      <c r="H30" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>5</v>
-      </c>
-      <c r="H31" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>5</v>
-      </c>
-      <c r="H32" t="s">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>5</v>
+      </c>
+      <c r="I33" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>5</v>
-      </c>
-      <c r="H33" t="s">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>5</v>
+      </c>
+      <c r="I34" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>5</v>
-      </c>
-      <c r="H34" t="s">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>5</v>
+      </c>
+      <c r="I35" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>5</v>
-      </c>
-      <c r="H35" t="s">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>5</v>
+      </c>
+      <c r="I36" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>5</v>
-      </c>
-      <c r="H36" t="s">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>5</v>
+      </c>
+      <c r="I37" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>5</v>
-      </c>
-      <c r="H37" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>28</v>
       </c>
-      <c r="H38" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I38" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B39" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" t="s">
+        <v>46</v>
+      </c>
+      <c r="I39" t="s">
         <v>47</v>
       </c>
-      <c r="H39" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>50</v>
       </c>
-      <c r="F40" t="s">
+      <c r="B40" t="s">
+        <v>57</v>
+      </c>
+      <c r="G40" t="s">
         <v>51</v>
       </c>
-      <c r="H40" t="s">
-        <v>49</v>
+      <c r="I40" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" t="s">
+        <v>57</v>
+      </c>
+      <c r="F41" t="s">
+        <v>53</v>
+      </c>
+      <c r="I41" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" t="s">
+        <v>58</v>
+      </c>
+      <c r="I42" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implements before pseudo to cause effect on timeline matching other games
</commit_message>
<xml_diff>
--- a/content/timeline.xlsx
+++ b/content/timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernardo.bozo/Desktop/Github/_THREEJS/LOK_timeline/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{CD360685-54F8-B545-8DB8-BE15B30DE299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2C8CAAB6-7D49-C34F-B952-50D3D01019C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="25100" xr2:uid="{7240041B-6A59-8449-9726-667E954DD1D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="64">
   <si>
     <t>class</t>
   </si>
@@ -185,9 +185,6 @@
     <t>Kain assassinates the young King William the Just, who will become the Nemesis</t>
   </si>
   <si>
-    <t>timeline-1 time-travel tt1</t>
-  </si>
-  <si>
     <t xml:space="preserve">timeline-1 time-travel </t>
   </si>
   <si>
@@ -216,6 +213,21 @@
   </si>
   <si>
     <t>Janos Audron is executed and his heart ripped from his body</t>
+  </si>
+  <si>
+    <t>The Corruption of the Pillars</t>
+  </si>
+  <si>
+    <t>Mortanius, the Guardian of Death, is possessed by a dark entity</t>
+  </si>
+  <si>
+    <t>Ariel, the Guardian of Balance, is murdered; the human Kain is born, destined to take her place</t>
+  </si>
+  <si>
+    <t>Ariel's murder drives her beloved, Nupraptor (the Pillar of the Mind), insane with grief. In his agony, he unleashes a telepathic assault which ripples across the Land of Nosgoth, infecting the other members of the Circle (who are all symbiotically connected) with his madness.</t>
+  </si>
+  <si>
+    <t>timeline-1 time-travel tt1 event</t>
   </si>
 </sst>
 </file>
@@ -602,7 +614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3815DBE4-1426-494D-8B3F-8B9461315769}">
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="23.33203125" customWidth="1"/>
@@ -614,7 +626,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>45</v>
@@ -905,7 +917,7 @@
         <v>5</v>
       </c>
       <c r="I31" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
@@ -966,10 +978,10 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="B39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C39" t="s">
         <v>46</v>
@@ -980,13 +992,13 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" t="s">
+        <v>56</v>
+      </c>
+      <c r="G40" t="s">
         <v>50</v>
-      </c>
-      <c r="B40" t="s">
-        <v>57</v>
-      </c>
-      <c r="G40" t="s">
-        <v>51</v>
       </c>
       <c r="I40" t="s">
         <v>48</v>
@@ -994,27 +1006,71 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F41" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I41" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>53</v>
+      </c>
+      <c r="B42" t="s">
+        <v>57</v>
+      </c>
+      <c r="I42" t="s">
         <v>54</v>
       </c>
-      <c r="B42" t="s">
-        <v>58</v>
-      </c>
-      <c r="I42" t="s">
-        <v>55</v>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>5</v>
+      </c>
+      <c r="D43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I43" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>5</v>
+      </c>
+      <c r="B44" t="s">
+        <v>56</v>
+      </c>
+      <c r="I44" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>5</v>
+      </c>
+      <c r="B45" t="s">
+        <v>56</v>
+      </c>
+      <c r="I45" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>5</v>
+      </c>
+      <c r="B46" t="s">
+        <v>56</v>
+      </c>
+      <c r="I46" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>